<commit_message>
Send Mowbray & Rondebosch batch 2026-10-08-0050
</commit_message>
<xml_diff>
--- a/inbox/mowbray_rondebosch_batch.xlsx
+++ b/inbox/mowbray_rondebosch_batch.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="66">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -616,6 +616,9 @@
       <c r="D4" t="s">
         <v>43</v>
       </c>
+      <c r="G4" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
@@ -630,6 +633,9 @@
       <c r="D5" t="s">
         <v>44</v>
       </c>
+      <c r="G5" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
@@ -644,6 +650,9 @@
       <c r="D6" t="s">
         <v>45</v>
       </c>
+      <c r="G6" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
@@ -658,6 +667,9 @@
       <c r="D7" t="s">
         <v>46</v>
       </c>
+      <c r="G7" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
@@ -672,6 +684,9 @@
       <c r="D8" t="s">
         <v>47</v>
       </c>
+      <c r="G8" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
@@ -686,6 +701,9 @@
       <c r="D9" t="s">
         <v>48</v>
       </c>
+      <c r="G9" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
@@ -700,6 +718,9 @@
       <c r="D10" t="s">
         <v>49</v>
       </c>
+      <c r="G10" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
@@ -714,6 +735,9 @@
       <c r="D11" t="s">
         <v>50</v>
       </c>
+      <c r="G11" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
@@ -728,6 +752,9 @@
       <c r="D12" t="s">
         <v>51</v>
       </c>
+      <c r="G12" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
@@ -742,6 +769,9 @@
       <c r="D13" t="s">
         <v>52</v>
       </c>
+      <c r="G13" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
@@ -756,6 +786,9 @@
       <c r="D14" t="s">
         <v>53</v>
       </c>
+      <c r="G14" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
@@ -770,6 +803,9 @@
       <c r="D15" t="s">
         <v>54</v>
       </c>
+      <c r="G15" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
@@ -784,8 +820,11 @@
       <c r="D16" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="17" spans="1:4">
+      <c r="G16" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
       <c r="A17" t="s">
         <v>22</v>
       </c>
@@ -798,8 +837,11 @@
       <c r="D17" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="18" spans="1:4">
+      <c r="G17" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -812,8 +854,11 @@
       <c r="D18" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="19" spans="1:4">
+      <c r="G18" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
       <c r="A19" t="s">
         <v>24</v>
       </c>
@@ -826,8 +871,11 @@
       <c r="D19" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="20" spans="1:4">
+      <c r="G19" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
       <c r="A20" t="s">
         <v>25</v>
       </c>
@@ -840,8 +888,11 @@
       <c r="D20" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="21" spans="1:4">
+      <c r="G20" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
       <c r="A21" t="s">
         <v>26</v>
       </c>
@@ -854,8 +905,11 @@
       <c r="D21" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="22" spans="1:4">
+      <c r="G21" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
       <c r="A22" t="s">
         <v>27</v>
       </c>
@@ -868,8 +922,11 @@
       <c r="D22" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="23" spans="1:4">
+      <c r="G22" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
       <c r="A23" t="s">
         <v>28</v>
       </c>
@@ -882,8 +939,11 @@
       <c r="D23" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="24" spans="1:4">
+      <c r="G23" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
       <c r="A24" t="s">
         <v>29</v>
       </c>
@@ -896,8 +956,11 @@
       <c r="D24" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="25" spans="1:4">
+      <c r="G24" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
       <c r="A25" t="s">
         <v>30</v>
       </c>
@@ -909,6 +972,9 @@
       </c>
       <c r="D25" t="s">
         <v>64</v>
+      </c>
+      <c r="G25" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>